<commit_message>
Enhance date handling in Form1702ExImportService and add tests for spreadsheet uploads
</commit_message>
<xml_diff>
--- a/public/form-assets/1702-ex/1702-ex-import-template.xlsx
+++ b/public/form-assets/1702-ex/1702-ex-import-template.xlsx
@@ -1,20 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sample Data" sheetId="1" state="visible" r:id="rId1"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
+  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">openpyxl</dc:creator>
+  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-04-09T13:44:40Z</dcterms:created>
+  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-04-09T13:44:40Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="1">
@@ -124,7 +124,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -407,13 +407,28 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sample Data" sheetId="1" state="visible" r:id="rId1"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DJ1"/>
+  <dimension ref="A1:DR1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,512 +494,552 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>incorporation_date</t>
+          <t>incorporation_date_month</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>incorporation_date_day</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>incorporation_date_year</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>contact_number</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>email_address</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>deduction_method</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>legal_basis</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>investment_agency</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>registered_activity</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>effectivity_from</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>effectivity_to</t>
-        </is>
-      </c>
       <c r="V1" t="inlineStr">
         <is>
+          <t>effectivity_from_month</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>effectivity_from_day</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>effectivity_from_year</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>effectivity_to_month</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>effectivity_to_day</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>effectivity_to_year</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>tax_due</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>tax_credits</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>overpayment</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>penalty_compromise</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>total_amount_payable</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>number_of_attachments</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>sales_receipts_revenues_fees</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>sales_returns_allowances_discounts</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>net_sales_receipts_revenues_fees</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>cost_of_sales_services</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>gross_income_from_operation</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>other_income</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>total_gross_income</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>ordinary_allowable_itemized_deductions</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>special_allowable_itemized_deductions</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>total_itemized_deductions</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>osd</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>net_taxable_income_loss</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>tax_rate</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>prior_years_excess_credits</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>income_tax_payment_previous_quarters</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>creditable_tax_withheld_previous_quarters</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>creditable_tax_withheld_fourth_quarter</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>foreign_tax_credits</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>tax_paid_return_previously_filed</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>other_tax_credits_payments_1_description</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>other_tax_credits_payments_1_amount</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>other_tax_credits_payments_2_description</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>other_tax_credits_payments_2_amount</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>regular_income_tax_otherwise_due</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>special_allowable_itemized_deductions_tax_relief</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>total_tax_relief_availment</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>schedule1_amortizations</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>schedule1_bad_debts</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>schedule1_charitable_contributions</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>schedule1_depletion</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>schedule1_depreciation</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>schedule1_entertainment_amusement_recreation</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>schedule1_fringe_benefits</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>schedule1_interest</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>schedule1_losses</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>schedule1_pension_trusts</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>schedule1_rental</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>schedule1_research_development</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>schedule1_salaries_wages_allowances</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>schedule1_sss_gsis_philhealth_hdmf_other_contributions</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>schedule1_taxes_and_licenses</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>schedule1_transportation_and_travel</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>schedule1_janitorial_messengerial_services_amount</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>schedule1_professional_fees_amount</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>schedule1_security_services_amount</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>schedule1_other_d_description</t>
         </is>
       </c>
-      <c r="BV1" t="inlineStr">
+      <c r="CB1" t="inlineStr">
         <is>
           <t>schedule1_other_d_amount</t>
         </is>
       </c>
-      <c r="BW1" t="inlineStr">
+      <c r="CC1" t="inlineStr">
         <is>
           <t>schedule1_other_e_description</t>
         </is>
       </c>
-      <c r="BX1" t="inlineStr">
+      <c r="CD1" t="inlineStr">
         <is>
           <t>schedule1_other_e_amount</t>
         </is>
       </c>
-      <c r="BY1" t="inlineStr">
+      <c r="CE1" t="inlineStr">
         <is>
           <t>schedule1_other_f_description</t>
         </is>
       </c>
-      <c r="BZ1" t="inlineStr">
+      <c r="CF1" t="inlineStr">
         <is>
           <t>schedule1_other_f_amount</t>
         </is>
       </c>
-      <c r="CA1" t="inlineStr">
+      <c r="CG1" t="inlineStr">
         <is>
           <t>schedule1_other_g_description</t>
         </is>
       </c>
-      <c r="CB1" t="inlineStr">
+      <c r="CH1" t="inlineStr">
         <is>
           <t>schedule1_other_g_amount</t>
         </is>
       </c>
-      <c r="CC1" t="inlineStr">
+      <c r="CI1" t="inlineStr">
         <is>
           <t>schedule1_other_h_description</t>
         </is>
       </c>
-      <c r="CD1" t="inlineStr">
+      <c r="CJ1" t="inlineStr">
         <is>
           <t>schedule1_other_h_amount</t>
         </is>
       </c>
-      <c r="CE1" t="inlineStr">
+      <c r="CK1" t="inlineStr">
         <is>
           <t>schedule1_other_i_description</t>
         </is>
       </c>
-      <c r="CF1" t="inlineStr">
+      <c r="CL1" t="inlineStr">
         <is>
           <t>schedule1_other_i_amount</t>
         </is>
       </c>
-      <c r="CG1" t="inlineStr">
+      <c r="CM1" t="inlineStr">
         <is>
           <t>schedule1_total_ordinary_allowable_itemized_deductions</t>
         </is>
       </c>
-      <c r="CH1" t="inlineStr">
+      <c r="CN1" t="inlineStr">
         <is>
           <t>schedule2_item_1_description</t>
         </is>
       </c>
-      <c r="CI1" t="inlineStr">
+      <c r="CO1" t="inlineStr">
         <is>
           <t>schedule2_item_1_legal_basis</t>
         </is>
       </c>
-      <c r="CJ1" t="inlineStr">
+      <c r="CP1" t="inlineStr">
         <is>
           <t>schedule2_item_1_amount</t>
         </is>
       </c>
-      <c r="CK1" t="inlineStr">
+      <c r="CQ1" t="inlineStr">
         <is>
           <t>schedule2_item_2_description</t>
         </is>
       </c>
-      <c r="CL1" t="inlineStr">
+      <c r="CR1" t="inlineStr">
         <is>
           <t>schedule2_item_2_legal_basis</t>
         </is>
       </c>
-      <c r="CM1" t="inlineStr">
+      <c r="CS1" t="inlineStr">
         <is>
           <t>schedule2_item_2_amount</t>
         </is>
       </c>
-      <c r="CN1" t="inlineStr">
+      <c r="CT1" t="inlineStr">
         <is>
           <t>schedule2_item_3_description</t>
         </is>
       </c>
-      <c r="CO1" t="inlineStr">
+      <c r="CU1" t="inlineStr">
         <is>
           <t>schedule2_item_3_legal_basis</t>
         </is>
       </c>
-      <c r="CP1" t="inlineStr">
+      <c r="CV1" t="inlineStr">
         <is>
           <t>schedule2_item_3_amount</t>
         </is>
       </c>
-      <c r="CQ1" t="inlineStr">
+      <c r="CW1" t="inlineStr">
         <is>
           <t>schedule2_item_4_description</t>
         </is>
       </c>
-      <c r="CR1" t="inlineStr">
+      <c r="CX1" t="inlineStr">
         <is>
           <t>schedule2_item_4_legal_basis</t>
         </is>
       </c>
-      <c r="CS1" t="inlineStr">
+      <c r="CY1" t="inlineStr">
         <is>
           <t>schedule2_item_4_amount</t>
         </is>
       </c>
-      <c r="CT1" t="inlineStr">
+      <c r="CZ1" t="inlineStr">
         <is>
           <t>schedule2_total_special_allowable_itemized_deductions</t>
         </is>
       </c>
-      <c r="CU1" t="inlineStr">
+      <c r="DA1" t="inlineStr">
         <is>
           <t>schedule3_net_income_loss_per_books</t>
         </is>
       </c>
-      <c r="CV1" t="inlineStr">
+      <c r="DB1" t="inlineStr">
         <is>
           <t>schedule3_add_non_deductible_1_description</t>
         </is>
       </c>
-      <c r="CW1" t="inlineStr">
+      <c r="DC1" t="inlineStr">
         <is>
           <t>schedule3_add_non_deductible_1_amount</t>
         </is>
       </c>
-      <c r="CX1" t="inlineStr">
+      <c r="DD1" t="inlineStr">
         <is>
           <t>schedule3_add_non_deductible_2_description</t>
         </is>
       </c>
-      <c r="CY1" t="inlineStr">
+      <c r="DE1" t="inlineStr">
         <is>
           <t>schedule3_add_non_deductible_2_amount</t>
         </is>
       </c>
-      <c r="CZ1" t="inlineStr">
+      <c r="DF1" t="inlineStr">
         <is>
           <t>schedule3_total_items_1_to_3</t>
         </is>
       </c>
-      <c r="DA1" t="inlineStr">
+      <c r="DG1" t="inlineStr">
         <is>
           <t>schedule3_less_non_taxable_income_subject_final_tax_description</t>
         </is>
       </c>
-      <c r="DB1" t="inlineStr">
+      <c r="DH1" t="inlineStr">
         <is>
           <t>schedule3_less_non_taxable_income_subject_final_tax_amount</t>
         </is>
       </c>
-      <c r="DC1" t="inlineStr">
+      <c r="DI1" t="inlineStr">
         <is>
           <t>schedule3_less_non_taxable_income_subject_final_tax_other_description</t>
         </is>
       </c>
-      <c r="DD1" t="inlineStr">
+      <c r="DJ1" t="inlineStr">
         <is>
           <t>schedule3_less_non_taxable_income_subject_final_tax_other_amount</t>
         </is>
       </c>
-      <c r="DE1" t="inlineStr">
+      <c r="DK1" t="inlineStr">
         <is>
           <t>schedule3_special_deductions_description</t>
         </is>
       </c>
-      <c r="DF1" t="inlineStr">
+      <c r="DL1" t="inlineStr">
         <is>
           <t>schedule3_special_deductions_amount</t>
         </is>
       </c>
-      <c r="DG1" t="inlineStr">
+      <c r="DM1" t="inlineStr">
         <is>
           <t>schedule3_special_deductions_other_description</t>
         </is>
       </c>
-      <c r="DH1" t="inlineStr">
+      <c r="DN1" t="inlineStr">
         <is>
           <t>schedule3_special_deductions_other_amount</t>
         </is>
       </c>
-      <c r="DI1" t="inlineStr">
+      <c r="DO1" t="inlineStr">
         <is>
           <t>schedule3_total_items_5_to_8</t>
         </is>
       </c>
-      <c r="DJ1" t="inlineStr">
+      <c r="DP1" t="inlineStr">
         <is>
           <t>schedule3_net_taxable_income_loss</t>
+        </is>
+      </c>
+      <c r="DQ1" t="inlineStr">
+        <is>
+          <t>client_name</t>
+        </is>
+      </c>
+      <c r="DR1" t="inlineStr">
+        <is>
+          <t>recipient</t>
         </is>
       </c>
     </row>

</xml_diff>